<commit_message>
Manejo de Fechas leídas de Excel actualizado
</commit_message>
<xml_diff>
--- a/TallerII/morosos.xlsx
+++ b/TallerII/morosos.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro\OneDrive\Documentos\GitHub\TallerII\TallerII\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39C5F3E-35BC-4EA1-82DA-41AF89905DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>ID</t>
   </si>
@@ -49,15 +55,6 @@
     <t>Luis Fernández</t>
   </si>
   <si>
-    <t>juan@escuela.edu.ar</t>
-  </si>
-  <si>
-    <t>maria@escuela.edu.ar</t>
-  </si>
-  <si>
-    <t>luis@escuela.edu.ar</t>
-  </si>
-  <si>
     <t>El Principito</t>
   </si>
   <si>
@@ -67,20 +64,56 @@
     <t>Don Quijote de la Mancha</t>
   </si>
   <si>
-    <t>2025-04-20</t>
-  </si>
-  <si>
-    <t>2025-04-18</t>
-  </si>
-  <si>
-    <t>2025-04-15</t>
+    <t>1004</t>
+  </si>
+  <si>
+    <t>1005</t>
+  </si>
+  <si>
+    <t>1006</t>
+  </si>
+  <si>
+    <t>juan@gmail.com</t>
+  </si>
+  <si>
+    <t>maria@gmail.com</t>
+  </si>
+  <si>
+    <t>luis@gmail.com</t>
+  </si>
+  <si>
+    <t>Alberto Silveira</t>
+  </si>
+  <si>
+    <t>albertito123@gmail.com</t>
+  </si>
+  <si>
+    <t>"1984"</t>
+  </si>
+  <si>
+    <t>Pablo Menoni</t>
+  </si>
+  <si>
+    <t>pablotacua@gmail.com</t>
+  </si>
+  <si>
+    <t>El archivo de las tormentas</t>
+  </si>
+  <si>
+    <t>Santiago Urioste</t>
+  </si>
+  <si>
+    <t>elchapita123@gmail.com</t>
+  </si>
+  <si>
+    <t>Arsené Lupin</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -92,6 +125,20 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -129,25 +176,65 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{09266A4F-3FF3-439B-97CF-4EB83BAA620F}">
+      <tableStyleElement type="wholeTable" dxfId="1"/>
+      <tableStyleElement type="headerRow" dxfId="0"/>
+    </tableStyle>
+  </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -189,7 +276,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -221,9 +308,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -255,6 +360,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -430,11 +553,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" customWidth="1"/>
+    <col min="3" max="3" width="29.85546875" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="21.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -451,58 +581,118 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" t="s">
-        <v>17</v>
+      <c r="E2" s="2">
+        <v>45950</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>18</v>
+      <c r="E3" s="2">
+        <v>45948</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" s="2">
+        <v>45945</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="2">
+        <v>45790</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="2">
+        <v>45791</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>16</v>
       </c>
-      <c r="E4" t="s">
-        <v>19</v>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="2">
+        <v>45792</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{EE6327AB-0582-44E5-8983-CEB8D85D8732}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{E506C4B6-0382-4C35-95B4-D30F4D3463FB}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{754D2E11-E9E1-4F14-B917-845A922770E5}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{E196DA11-95E5-4F71-913E-B346ECA75903}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{13F38172-CF64-4415-882A-4FE7FCB49AA6}"/>
+    <hyperlink ref="C7" r:id="rId6" xr:uid="{A75146C2-C4FE-4EF7-92DE-F7CEF0F4CB5E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>